<commit_message>
v2 - changed the db logic
</commit_message>
<xml_diff>
--- a/templates/EXP_TEMPLET.xlsx
+++ b/templates/EXP_TEMPLET.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="6"/>
+    <workbookView firstSheet="6" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="ITEM" sheetId="1"/>
@@ -576,9 +576,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
-    <numFmt numFmtId="15571" formatCode="0.00;[Red]0.00"/>
-    <numFmt numFmtId="15572" formatCode="0.000;[Red]0.000"/>
-    <numFmt numFmtId="15573" formatCode="0.00000;[Red]0.00000"/>
+    <numFmt numFmtId="10951" formatCode="0.00;[Red]0.00"/>
+    <numFmt numFmtId="10952" formatCode="0.000;[Red]0.000"/>
+    <numFmt numFmtId="10953" formatCode="0.00000;[Red]0.00000"/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -1113,13 +1113,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15571" fontId="0" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="10951" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15572" fontId="0" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="10952" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15573" fontId="0" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="10953" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="34" borderId="10" xfId="38">
@@ -1505,7 +1505,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{31531CC8-74D7-4F20-8903-50552658ED35}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D65A7104-92B6-43A2-A393-7A8F1EAA5F71}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:AS118"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -11411,7 +11411,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DCA1E4F2-5FEC-4B17-8A41-210798983AF8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{ED3619CA-2E97-4814-990C-C59AABC32BA1}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -11465,7 +11465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{12DF8B69-49C1-4B4F-8A04-A22D2C7F496F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6F1B0258-09FD-44AE-AB9D-BA91391BE43A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -11520,7 +11520,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0DDD3292-5A5A-4C3A-812B-FBFC3FF67EED}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{34A0BD87-3CE8-4021-8B54-EBC571758037}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -11574,7 +11574,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1135453D-BD55-4419-9DA1-027AF28C22B2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A3B22773-8E8D-46E2-9386-388E08A290F8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:X1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -11688,7 +11688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{71098884-ADBC-4444-8D6C-59E85BA5C56C}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{662C4981-4EAB-46B4-BB1D-E5A35D3139D9}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:D118"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13013,7 +13013,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4A5CBC8C-20F4-4A07-95BD-BAEC7ED71CD8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{7E2D4AEB-C8C2-4B21-A93D-D0F4017E8FCF}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13086,7 +13086,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3AC212B7-1287-414B-8C7B-B2161D3E6D02}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5CFEBA6C-F6AA-4ADF-8C41-857223366C0F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13123,7 +13123,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B3902A4A-55F5-4713-AC9C-EC7B577F8ADB}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DFE66705-1C25-4505-A992-C9B331DF3452}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13180,7 +13180,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{98FCD8B6-1CE1-43E1-921F-33B459523D3F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{37EF2289-E4FE-484D-B147-5977322EC9F4}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13211,7 +13211,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{22B75733-77CB-4764-B13D-9B12DFBA5FB8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1F3DD609-B3D9-48D3-B42C-8E8D77B95212}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13273,7 +13273,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8B585255-2018-4D36-B81A-70726DF02B01}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5E042E26-70FC-4AF2-B38B-44DFDF093DD2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -13338,7 +13338,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{254FD3BD-DB3C-459B-A74C-70F669CE319A}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1B8FEEBC-5A7E-47BF-AE03-A92113A0B088}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="12.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>

</xml_diff>